<commit_message>
Pull the origination scanner's TRACKER history into the daily workbook (tab 9 - Track Record). track_record.py reads recommendations_log.csv (406 picks since 7/1), snapshots it, and scores by grade and tab. CRITICAL: cur_ret/best_ret/worst_ret are FRACTIONS - x100. First read is honest and unflattering: 406 picks 39pct green, mean -2.16pct over ~8 days in a flat July tape = underperforming; grade adds NO edge (A -2.78pct vs B -2.02pct, higher grade did worse); score does not predict (top-25pct vs bottom-25pct spread -0.60pt, backwards) - the SAME verdict as the BUY SCORE calibration, now two independent scores both failing to rank returns. All still OPEN (log started 7/1, nothing at 21d yet) so these are unrealized reads, real win-rates land through early August. Tab formatted consistent (tooltips all cols, mean-return colouring). Renumbered Data Quality to 10, Run Summary to 11.
</commit_message>
<xml_diff>
--- a/reports/universe_2026-07-22_new.xlsx
+++ b/reports/universe_2026-07-22_new.xlsx
@@ -16,8 +16,9 @@
     <sheet name="6 - Tracker Broken" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="7 - Notes &amp; Decisions" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="8 - Market Movers" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="9 - Data Quality" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="10 - Run Summary" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="9 - Track Record" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="10 - Data Quality" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="11 - Run Summary" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2 - Fresh Buys'!$A$1:$W$1</definedName>
@@ -27,7 +28,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6 - Tracker Broken'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'7 - Notes &amp; Decisions'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'8 - Market Movers'!$A$1:$I$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'9 - Data Quality'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'10 - Data Quality'!$A$1:$E$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -107,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -175,6 +176,15 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -281,6 +291,46 @@
 </file>
 
 <file path=xl/comments/comment10.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>scan</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>BLOCKER = this run's conclusions may be WRONG until fixed. WARNING = a real limitation, read before acting. INFO = context.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Which part of the pipeline the issue is in.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>The problem, stated plainly in one or two sentences.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>What this actually means for the numbers in this workbook - which conclusions you can and cannot trust.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>The concrete fix or the check to run before trusting this again.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment11.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>scan</author>
@@ -830,31 +880,43 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>BLOCKER = this run's conclusions may be WRONG until fixed. WARNING = a real limitation, read before acting. INFO = context.
+        <t>The pick group being scored - all picks, then by grade, then by origination tab.
 (Full guide: 'READ ME FIRST' tab)</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Which part of the pipeline the issue is in.
+        <t>How many recommendations in this group.
 (Full guide: 'READ ME FIRST' tab)</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>The problem, stated plainly in one or two sentences.
+        <t>Share currently in profit (unrealized).
 (Full guide: 'READ ME FIRST' tab)</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>What this actually means for the numbers in this workbook - which conclusions you can and cannot trust.
+        <t>Average unrealized return since the pick.
 (Full guide: 'READ ME FIRST' tab)</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>The concrete fix or the check to run before trusting this again.
+        <t>Median - less distorted by outliers.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Average best excursion reached - upside that was on the table.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Average worst drawdown suffered - pain held through.
 (Full guide: 'READ ME FIRST' tab)</t>
       </text>
     </comment>
@@ -1151,7 +1213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1201,7 +1263,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22 19:16 local</t>
+          <t>2026-07-22 21:29 local</t>
         </is>
       </c>
     </row>
@@ -1422,12 +1484,12 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>9 - Data Quality</t>
+          <t>9 - Track Record</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>What was broken or partial in this run, ranked by severity.</t>
+          <t>How the scanner's past picks have actually done - the honest scorecard.</t>
         </is>
       </c>
     </row>
@@ -1435,54 +1497,58 @@
       <c r="A31" t="inlineStr"/>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">    READ THE RED ROWS. A BLOCKER means conclusions in this file may be wrong.</t>
+          <t xml:space="preserve">    Broken down by grade and tab; shows whether a higher grade is worth more (so far, no).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>10 - Run Summary</t>
+          <t>10 - Data Quality</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
+          <t>What was broken or partial in this run, ranked by severity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    READ THE RED ROWS. A BLOCKER means conclusions in this file may be wrong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>11 - Run Summary</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
           <t>Counts and run metadata.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="B33" s="2" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="35">
+      <c r="B35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>HOW TO ACT ON IT</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr"/>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>1. Check tab 9 for BLOCKERS first. If coverage was partial, absence of a name</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr"/>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   proves nothing - it may simply never have been scanned.</t>
-        </is>
-      </c>
+      <c r="B36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>2. Read the regime on tab 1. It sets your size for everything else.</t>
+          <t>1. Check tab 10 for BLOCKERS first. If coverage was partial, absence of a name</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1556,7 @@
       <c r="A38" t="inlineStr"/>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>3. Work tab 2 top-down. Only green Verdicts are candidates.</t>
+          <t xml:space="preserve">   proves nothing - it may simply never have been scanned.</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1564,7 @@
       <c r="A39" t="inlineStr"/>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>4. Cross-check each candidate against tab 5 - a sell-mode name is never a buy.</t>
+          <t>2. Read the regime on tab 1. It sets your size for everything else.</t>
         </is>
       </c>
     </row>
@@ -1506,88 +1572,104 @@
       <c r="A40" t="inlineStr"/>
       <c r="B40" s="2" t="inlineStr">
         <is>
+          <t>3. Work tab 2 top-down. Only green Verdicts are candidates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>4. Cross-check each candidate against tab 5 - a sell-mode name is never a buy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
           <t>5. Size it on tab 3. If the stop is wider than the risk unit allows, skip it.</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="B41" s="2" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+    <row r="43">
+      <c r="B43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>WHAT THE NUMBERS MEAN</t>
         </is>
       </c>
-      <c r="B42" s="2" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>Magical (CCI-20)</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Above +100 = overbought, below -100 = oversold. NOTE: measured 2026-07-22 across 1,725 signals, this cut does NOT separate returns (0.03pt over 21 days). Treat as context, not a veto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>ZLSMA-50</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>The trend line. Price below it on a buy signal is a structural fail.</t>
-        </is>
-      </c>
+      <c r="B44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Chandelier Exit</t>
+          <t>Magical (CCI-20)</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Flips BUY/SELL. The label price is the STOP level, not an entry.</t>
+          <t>Above +100 = overbought, below -100 = oversold. NOTE: measured 2026-07-22 across 1,725 signals, this cut does NOT separate returns (0.03pt over 21 days). Treat as context, not a veto.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>Regime PASS</t>
+          <t>ZLSMA-50</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Above a rising 200-day and beating SPY -&gt; normal size.</t>
+          <t>The trend line. Price below it on a buy signal is a structural fail.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Regime REPAIR</t>
+          <t>Chandelier Exit</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Below the 200-day -&gt; starter size only.</t>
+          <t>Flips BUY/SELL. The label price is the STOP level, not an entry.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
+          <t>Regime PASS</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Above a rising 200-day and beating SPY -&gt; normal size.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Regime REPAIR</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Below the 200-day -&gt; starter size only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
           <t>Regime DEEP-FAIL</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>More than 10% below the 200-day -&gt; watch only, no size.</t>
         </is>
@@ -1599,6 +1681,295 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Picks</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Green %</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Mean Return %</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Median Return %</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Avg Best %</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Avg Worst %</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>ALL PICKS</t>
+        </is>
+      </c>
+      <c r="B2" s="26" t="n">
+        <v>406</v>
+      </c>
+      <c r="C2" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="D2" s="10" t="n">
+        <v>-2.16</v>
+      </c>
+      <c r="E2" s="10" t="n">
+        <v>-0.99</v>
+      </c>
+      <c r="F2" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" s="10" t="n">
+        <v>-7.4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>grade A+</t>
+        </is>
+      </c>
+      <c r="B3" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="15" t="n">
+        <v>50</v>
+      </c>
+      <c r="D3" s="15" t="n">
+        <v>-10.87</v>
+      </c>
+      <c r="E3" s="15" t="n">
+        <v>-10.87</v>
+      </c>
+      <c r="F3" s="15" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="G3" s="15" t="n">
+        <v>-22.1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>grade A</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="D4" s="19" t="n">
+        <v>-2.78</v>
+      </c>
+      <c r="E4" s="19" t="n">
+        <v>-1.34</v>
+      </c>
+      <c r="F4" s="19" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="G4" s="19" t="n">
+        <v>-9.300000000000001</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>grade B</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="n">
+        <v>354</v>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>38</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>-2.02</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>-0.96</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>tab BUY ZONE</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="n">
+        <v>24</v>
+      </c>
+      <c r="C6" s="19" t="n">
+        <v>38</v>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>-0.71</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>-8.6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>tab COILED</t>
+        </is>
+      </c>
+      <c r="B7" s="28" t="n">
+        <v>151</v>
+      </c>
+      <c r="C7" s="19" t="n">
+        <v>42</v>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>-1.21</v>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>-0.47</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <v>-5.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>tab COOLING</t>
+        </is>
+      </c>
+      <c r="B8" s="27" t="n">
+        <v>189</v>
+      </c>
+      <c r="C8" s="15" t="n">
+        <v>35</v>
+      </c>
+      <c r="D8" s="15" t="n">
+        <v>-3.47</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>-2.02</v>
+      </c>
+      <c r="F8" s="15" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>-9.199999999999999</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>tab FRESH IGNITION</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="n">
+        <v>42</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>-0.17</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>-6.3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>ORIGINATION SCANNER TRACK RECORD - 406 picks, 2026-07-01 to 2026-07-22. Returns are UNREALIZED (matured 0/406 at the 21-day mark; the log only started 7/1). This grades the scanner's own A/B/C picks, separate from the trade-call ledger.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>DOES THE SCORE PREDICT? bottom-25% by score mean -2.21%, top-25% mean -2.81%, spread -0.60pt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>The origination score does NOT predict returns here - flat/backwards, the SAME result as the BUY SCORE calibration. Two independent scores, same verdict: sort what to look at, do not forecast.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Unrealized reads on OPEN positions, not final results. Grade A (mean -2.8%) is NOT beating grade B (-2.0%) - higher grade has not paid so far. Real win-rates land as the July picks reach 21 days through early August.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1717,7 +2088,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1774,7 +2145,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>2026-07-22 19:16 local</t>
+          <t>2026-07-22 21:29 local</t>
         </is>
       </c>
     </row>

</xml_diff>